<commit_message>
Update API inventory to reflect runtime verification
Add runtime verification results to the API inventory, confirming 108 endpoints.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 8d464111-5c3e-47b3-aa90-797c0866066c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 863eb864-583a-4ca3-a7b7-1627626dc35d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0bd4c247-9f4d-4d27-aae0-8568e44e9555/8d464111-5c3e-47b3-aa90-797c0866066c/0T6VjA0
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/api-inventory.xlsx
+++ b/exports/api-inventory.xlsx
@@ -11,6 +11,7 @@
     <sheet name="By Feature" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Load Test Priorities" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Middleware &amp; Auth" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Runtime Verification" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4851,6 +4852,174 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>/api/twitter/retest</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>routes/twitter.ts</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>inline handler</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Clerk session cookie</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Re-verify X connection</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Social: X</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>/api/linkedin/retest</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>routes/linkedin.ts</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>inline handler</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Clerk session cookie</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Re-verify LinkedIn connection</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Social: LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>/api/youtube/retest</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>routes/youtube.ts</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>inline handler</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Clerk session cookie</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Re-verify YouTube connection</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Social: YouTube</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>/api/threads/retest</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>routes/threads.ts</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>inline handler</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Clerk session cookie</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Re-verify Threads connection</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Social: Threads</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4862,7 +5031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E105"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -7704,6 +7873,114 @@
       <c r="E105" t="inlineStr">
         <is>
           <t>Health check / liveness probe</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Social: X</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>/api/twitter/retest</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Re-verify X connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Social: LinkedIn</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>/api/linkedin/retest</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Re-verify LinkedIn connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Social: YouTube</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>/api/youtube/retest</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Re-verify YouTube connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Social: Threads</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>/api/threads/retest</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Re-verify Threads connection</t>
         </is>
       </c>
     </row>
@@ -8085,4 +8362,178 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GET /api/healthz (no auth)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>200 OK — public confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GET /api/plans (no auth)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>200 OK — public confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GET /api/app-brand (no auth)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>200 OK — public confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GET /api/me,/content,/accounts,/schedules,/notifications,/brand-kits without session</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>401 — auth gate (requireTenant) confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GET /api/admin/stats without session</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>401 — admin routes behind the same auth gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GET /api/twitter/auth/callback without valid state</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>302 redirect (safe error redirect) — reachable but protected by HMAC state</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>POST /api/*/retest without session (4 platforms)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>401 — routes exist and are auth-gated (missed in first static scan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Live frontend traffic observed in server logs</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GET /api/app-brand, /api/me, /api/content, /api/schedules, /api/notifications — matches inventory; all frontend calls go through generated hooks</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OpenAPI spec vs code</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>78 spec paths, all map 1:1 to code routes; no spec-only or code-only endpoints remain after adding the 4 retest routes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Unreachable/unused endpoints</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>None found. Every route is mounted in routes/index.ts and has a frontend or mobile caller; connection sweep also calls retest logic internally</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>New: mobile app (artifacts/mobile)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Second API consumer — uses bearer tokens (Clerk session token via Authorization header) instead of cookies</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Final count</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>108 endpoints (104 original + 4 platform retest routes)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>